<commit_message>
feat: publish audience reports atomically
</commit_message>
<xml_diff>
--- a/examples/strict-excel-project/DCC-cleaning-plan.xlsx
+++ b/examples/strict-excel-project/DCC-cleaning-plan.xlsx
@@ -4975,7 +4975,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" bestFit="1" customWidth="1" hidden="false" width="26.711"/>
@@ -5045,25 +5045,67 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>include_audit_report</t>
+          <t>include_statistical_report</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
           <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>include_machine_report</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>statistical_table_format</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>parquet</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>include_sensitive_examples</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>FALSE</t>
         </is>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1"/>
-  <dataValidations count="3">
+  <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3" errorStyle="stop" errorTitle="请选择有效值 / Choose a value" error="zh-CN, en" promptTitle="请选择有效值 / Choose a value" prompt="zh-CN, en">
       <formula1>"zh-CN,en"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B4" errorStyle="stop" errorTitle="请选择有效值 / Choose a value" error="csv, xlsx, parquet" promptTitle="请选择有效值 / Choose a value" prompt="csv, xlsx, parquet">
       <formula1>"csv,xlsx,parquet"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5:B6" errorStyle="stop" errorTitle="请选择有效值 / Choose a value" error="TRUE, FALSE" promptTitle="请选择有效值 / Choose a value" prompt="TRUE, FALSE">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5:B7" errorStyle="stop" errorTitle="请选择有效值 / Choose a value" error="TRUE, FALSE" promptTitle="请选择有效值 / Choose a value" prompt="TRUE, FALSE">
+      <formula1>"TRUE,FALSE"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8" errorStyle="stop" errorTitle="请选择有效值 / Choose a value" error="parquet, csv" promptTitle="请选择有效值 / Choose a value" prompt="parquet, csv">
+      <formula1>"parquet,csv"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B9" errorStyle="stop" errorTitle="请选择有效值 / Choose a value" error="TRUE, FALSE" promptTitle="请选择有效值 / Choose a value" prompt="TRUE, FALSE">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>